<commit_message>
Improve Excel pagination and cell layout with large conversion examples
Paginate wide ranges horizontally after bounded scaling, preserve per-page coordinates, and improve cell text overflow and stacked text rendering. Add reproducible 120-column by 300-row examples and refresh API documentation. Improve Azurite startup diagnostics for local launchers.

Validation: 85 Java tests passed; local-launcher tests passed with Windows-only cases skipped on macOS; 12 real HTTP conversions succeeded; API Docs build passed.
</commit_message>
<xml_diff>
--- a/docs/APIDocs/excel2img/examples/additional/inputs/embedded-images.xlsx
+++ b/docs/APIDocs/excel2img/examples/additional/inputs/embedded-images.xlsx
@@ -7,12 +7,18 @@
   </bookViews>
   <sheets>
     <sheet name="画像3種と記録" r:id="rId3" sheetId="1"/>
+    <sheet name="文字のはみ出し比較" r:id="rId4" sheetId="2"/>
+    <sheet name="縦書きと折返し中央" r:id="rId5" sheetId="3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">文字のはみ出し比較!$A$1:$L$22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">縦書きと折返し中央!$A$1:$U$26</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="51">
   <si>
     <t/>
   </si>
@@ -87,6 +93,100 @@
   <si>
     <t>画像は外部から取得せず、この生成スクリプトが作成したテスト用PNGです。
 このシートには印刷範囲を設定せず、セルと画像の使用範囲が自動選択されることも確認します。</t>
+  </si>
+  <si>
+    <t>セル文字の表示比較 / プログラム名</t>
+  </si>
+  <si>
+    <t>同じ文字を、狭い単独セル・結合セル・隣に値があるセルで比較します。
+ラベルは14pt、左寄せ、折り返しなしです。塗りつぶし済みの空セルにも文字が続くことを確認します。</t>
+  </si>
+  <si>
+    <t>① 狭いC8 + 同色の空セルD8:E8 / ラベル全体が見える</t>
+  </si>
+  <si>
+    <t>プログラム名</t>
+  </si>
+  <si>
+    <t>D8・E8は値なしの空セル。
+C8の文字が右へ続くことを確認します。</t>
+  </si>
+  <si>
+    <t>② C13:E13の結合セル / 同じラベル全体が見える</t>
+  </si>
+  <si>
+    <t>結合範囲の幅を使って表示します。
+①と②で文字が欠けないことを比較します。</t>
+  </si>
+  <si>
+    <t>③ 狭いC18 + D18に値あり / 隣の値へ侵入しない</t>
+  </si>
+  <si>
+    <t>隣の値</t>
+  </si>
+  <si>
+    <t>D18には文字列があります。
+C18のラベルはセル境界で止まり、隣の値を覆いません。</t>
+  </si>
+  <si>
+    <t>セル参照：はみ出し C8→D8:E8 / 結合 C13:E13 / 停止 C18→値ありD18。
+いずれも架空の表示確認用ラベルです。</t>
+  </si>
+  <si>
+    <t>ウィンドウ</t>
+  </si>
+  <si>
+    <t>検証結果</t>
+  </si>
+  <si>
+    <t>写真だけではセル書式を断定せず、縦書き255と折り返し＋上下左右中央揃えを比較します。
+各見出しは縦長の結合セルです。①は上揃え、②③は中央揃えで、幅も変えています。</t>
+  </si>
+  <si>
+    <t>① 縦書き255</t>
+  </si>
+  <si>
+    <t>② 折返し中央・1字幅</t>
+  </si>
+  <si>
+    <t>③ 折返し中央・2字幅</t>
+  </si>
+  <si>
+    <t>起動</t>
+  </si>
+  <si>
+    <t>表示内容</t>
+  </si>
+  <si>
+    <t>表示順</t>
+  </si>
+  <si>
+    <t>検索機能</t>
+  </si>
+  <si>
+    <t>PG検証</t>
+  </si>
+  <si>
+    <t>カーソル移動順</t>
+  </si>
+  <si>
+    <t>CENTER / TOP
+rotation=255
+縦方向の文字送り</t>
+  </si>
+  <si>
+    <t>CENTER / CENTER
+wrapText=true
+約1文字幅で折り返し</t>
+  </si>
+  <si>
+    <t>CENTER / CENTER
+wrapText=true
+約2文字幅で折り返し</t>
+  </si>
+  <si>
+    <t>確認する文字：起動 / 表示内容 / 表示順 / 検索機能 / PG検証 / カーソル移動順。
+縦書きと自動折り返しは異なるExcel書式です。文字の並び、中央位置、欠けを比較します。</t>
   </si>
 </sst>
 </file>
@@ -94,7 +194,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -148,6 +248,29 @@
     <font>
       <name val="BIZ UDPGothic"/>
       <sz val="11.0"/>
+      <b val="true"/>
+      <color rgb="FF1B2F41"/>
+    </font>
+    <font>
+      <name val="BIZ UDPGothic"/>
+      <sz val="14.0"/>
+      <b val="true"/>
+      <color rgb="FF1B2F41"/>
+    </font>
+    <font>
+      <name val="BIZ UDPGothic"/>
+      <sz val="11.0"/>
+      <color rgb="FF1B2F41"/>
+    </font>
+    <font>
+      <name val="BIZ UDPGothic"/>
+      <sz val="14.0"/>
+      <b val="true"/>
+      <color rgb="FF1B2F41"/>
+    </font>
+    <font>
+      <name val="BIZ UDPGothic"/>
+      <sz val="14.0"/>
       <b val="true"/>
       <color rgb="FF1B2F41"/>
     </font>
@@ -304,7 +427,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="true" applyAlignment="true" applyFill="true">
       <alignment wrapText="true" vertical="center"/>
@@ -332,6 +455,18 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyFont="true" applyAlignment="true" applyFill="true">
       <alignment wrapText="true" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" xfId="0" applyFont="true" applyAlignment="true" applyFill="true">
+      <alignment wrapText="false" vertical="center" horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyFont="true" applyAlignment="true" applyFill="true">
+      <alignment wrapText="false" vertical="center" horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="8" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment wrapText="false" vertical="top" textRotation="255" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="8" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment wrapText="true" vertical="center" textRotation="0" horizontal="center"/>
     </xf>
   </cellXfs>
 </styleSheet>
@@ -1126,4 +1261,1950 @@
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L22"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="10.0" customWidth="true"/>
+    <col min="2" max="2" width="10.0" customWidth="true"/>
+    <col min="3" max="3" width="5.0" customWidth="true"/>
+    <col min="4" max="4" width="9.0" customWidth="true"/>
+    <col min="5" max="5" width="9.0" customWidth="true"/>
+    <col min="6" max="6" width="10.0" customWidth="true"/>
+    <col min="7" max="7" width="10.0" customWidth="true"/>
+    <col min="8" max="8" width="10.0" customWidth="true"/>
+    <col min="9" max="9" width="10.0" customWidth="true"/>
+    <col min="10" max="10" width="10.0" customWidth="true"/>
+    <col min="11" max="11" width="10.0" customWidth="true"/>
+    <col min="12" max="12" width="10.0" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28.0" customHeight="true">
+      <c r="A1" t="s" s="1">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="H1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="J1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="K1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="L1" t="s" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" ht="28.0" customHeight="true">
+      <c r="A2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="L2" t="s" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" ht="28.0" customHeight="true">
+      <c r="A3" t="s" s="8">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L3" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="28.0" customHeight="true">
+      <c r="A4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="E4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="F4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L4" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="28.0" customHeight="true"/>
+    <row r="6" ht="28.0" customHeight="true">
+      <c r="A6" t="s" s="2">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="F6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="I6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="J6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="K6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="L6" t="s" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="28.0" customHeight="true"/>
+    <row r="8" ht="28.0" customHeight="true">
+      <c r="C8" t="s" s="10">
+        <v>27</v>
+      </c>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="G8" t="s" s="8">
+        <v>28</v>
+      </c>
+      <c r="H8" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I8" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J8" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K8" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L8" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="28.0" customHeight="true">
+      <c r="G9" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I9" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J9" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K9" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L9" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="28.0" customHeight="true"/>
+    <row r="11" ht="28.0" customHeight="true">
+      <c r="A11" t="s" s="2">
+        <v>29</v>
+      </c>
+      <c r="B11" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="C11" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="F11" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="G11" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="I11" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="J11" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="K11" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="L11" t="s" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="28.0" customHeight="true"/>
+    <row r="13" ht="28.0" customHeight="true">
+      <c r="C13" t="s" s="10">
+        <v>27</v>
+      </c>
+      <c r="D13" t="s" s="10">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s" s="10">
+        <v>0</v>
+      </c>
+      <c r="G13" t="s" s="8">
+        <v>30</v>
+      </c>
+      <c r="H13" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I13" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J13" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K13" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L13" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="28.0" customHeight="true">
+      <c r="G14" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H14" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I14" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J14" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K14" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L14" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="28.0" customHeight="true"/>
+    <row r="16" ht="28.0" customHeight="true">
+      <c r="A16" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="C16" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="D16" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="E16" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="F16" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="G16" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="H16" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="I16" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="J16" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="K16" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="L16" t="s" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="28.0" customHeight="true"/>
+    <row r="18" ht="28.0" customHeight="true">
+      <c r="C18" t="s" s="10">
+        <v>27</v>
+      </c>
+      <c r="D18" t="s" s="11">
+        <v>32</v>
+      </c>
+      <c r="E18" s="10"/>
+      <c r="G18" t="s" s="8">
+        <v>33</v>
+      </c>
+      <c r="H18" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I18" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J18" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K18" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L18" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="28.0" customHeight="true">
+      <c r="G19" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H19" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I19" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J19" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K19" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L19" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="28.0" customHeight="true"/>
+    <row r="21" ht="28.0" customHeight="true">
+      <c r="A21" t="s" s="8">
+        <v>34</v>
+      </c>
+      <c r="B21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="C21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="D21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="F21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="G21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L21" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="28.0" customHeight="true">
+      <c r="A22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="B22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="C22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="D22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="E22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="F22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="G22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L22" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="A3:L4"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="G8:L9"/>
+    <mergeCell ref="A11:L11"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="G13:L14"/>
+    <mergeCell ref="A16:L16"/>
+    <mergeCell ref="G18:L19"/>
+    <mergeCell ref="A21:L22"/>
+  </mergeCells>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U26"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="4.0" customWidth="true"/>
+    <col min="2" max="2" width="4.0" customWidth="true"/>
+    <col min="3" max="3" width="4.0" customWidth="true"/>
+    <col min="4" max="4" width="4.0" customWidth="true"/>
+    <col min="5" max="5" width="4.0" customWidth="true"/>
+    <col min="6" max="6" width="4.0" customWidth="true"/>
+    <col min="7" max="7" width="3.0" customWidth="true"/>
+    <col min="8" max="8" width="4.0" customWidth="true"/>
+    <col min="9" max="9" width="4.0" customWidth="true"/>
+    <col min="10" max="10" width="4.0" customWidth="true"/>
+    <col min="11" max="11" width="4.0" customWidth="true"/>
+    <col min="12" max="12" width="4.0" customWidth="true"/>
+    <col min="13" max="13" width="4.0" customWidth="true"/>
+    <col min="14" max="14" width="3.0" customWidth="true"/>
+    <col min="15" max="15" width="7.0" customWidth="true"/>
+    <col min="16" max="16" width="7.0" customWidth="true"/>
+    <col min="17" max="17" width="7.0" customWidth="true"/>
+    <col min="18" max="18" width="7.0" customWidth="true"/>
+    <col min="19" max="19" width="7.0" customWidth="true"/>
+    <col min="20" max="20" width="7.0" customWidth="true"/>
+    <col min="21" max="21" width="7.0" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24.0" customHeight="true">
+      <c r="A1" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="H1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="J1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="K1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="L1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="M1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="N1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="O1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="P1" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="Q1" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="R1" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="S1" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="T1" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="U1" t="s" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" ht="24.0" customHeight="true">
+      <c r="A2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="L2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="M2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="N2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="O2" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="P2" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="R2" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="S2" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="T2" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="U2" t="s" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" ht="30.0" customHeight="true">
+      <c r="A3" t="s" s="8">
+        <v>37</v>
+      </c>
+      <c r="B3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="M3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="N3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="O3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="P3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="R3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="S3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="T3" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="U3" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="30.0" customHeight="true">
+      <c r="A4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="E4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="F4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="M4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="N4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="O4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="P4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="R4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="S4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="T4" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="U4" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="24.0" customHeight="true"/>
+    <row r="6" ht="40.0" customHeight="true">
+      <c r="A6" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="B6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="F6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s" s="2">
+        <v>39</v>
+      </c>
+      <c r="I6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="J6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="K6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="L6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="M6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="O6" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="P6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="R6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="S6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="T6" t="s" s="2">
+        <v>0</v>
+      </c>
+      <c r="U6" t="s" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="24.0" customHeight="true">
+      <c r="A7" t="s" s="12">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s" s="12">
+        <v>42</v>
+      </c>
+      <c r="C7" t="s" s="12">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s" s="12">
+        <v>44</v>
+      </c>
+      <c r="E7" t="s" s="12">
+        <v>45</v>
+      </c>
+      <c r="F7" t="s" s="12">
+        <v>46</v>
+      </c>
+      <c r="H7" t="s" s="13">
+        <v>41</v>
+      </c>
+      <c r="I7" t="s" s="13">
+        <v>42</v>
+      </c>
+      <c r="J7" t="s" s="13">
+        <v>43</v>
+      </c>
+      <c r="K7" t="s" s="13">
+        <v>44</v>
+      </c>
+      <c r="L7" t="s" s="13">
+        <v>45</v>
+      </c>
+      <c r="M7" t="s" s="13">
+        <v>46</v>
+      </c>
+      <c r="O7" t="s" s="13">
+        <v>41</v>
+      </c>
+      <c r="P7" t="s" s="13">
+        <v>42</v>
+      </c>
+      <c r="Q7" t="s" s="13">
+        <v>43</v>
+      </c>
+      <c r="R7" t="s" s="13">
+        <v>44</v>
+      </c>
+      <c r="S7" t="s" s="13">
+        <v>45</v>
+      </c>
+      <c r="T7" t="s" s="13">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" ht="24.0" customHeight="true">
+      <c r="A8" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B8" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C8" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D8" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E8" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F8" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I8" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J8" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K8" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L8" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M8" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O8" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P8" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R8" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S8" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T8" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="24.0" customHeight="true">
+      <c r="A9" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B9" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C9" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D9" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F9" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I9" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J9" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K9" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L9" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M9" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O9" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P9" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R9" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S9" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T9" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="24.0" customHeight="true">
+      <c r="A10" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B10" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C10" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D10" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F10" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H10" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I10" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J10" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K10" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L10" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M10" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O10" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P10" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R10" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S10" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T10" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="24.0" customHeight="true">
+      <c r="A11" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B11" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C11" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F11" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I11" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J11" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K11" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L11" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M11" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O11" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P11" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R11" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S11" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T11" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="24.0" customHeight="true">
+      <c r="A12" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B12" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D12" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F12" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H12" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I12" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J12" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K12" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L12" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M12" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O12" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P12" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R12" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S12" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T12" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="24.0" customHeight="true">
+      <c r="A13" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B13" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C13" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D13" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F13" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H13" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I13" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J13" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K13" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L13" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M13" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O13" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P13" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R13" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S13" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T13" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="24.0" customHeight="true">
+      <c r="A14" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B14" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C14" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D14" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F14" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H14" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I14" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J14" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K14" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L14" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M14" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O14" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P14" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R14" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S14" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T14" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="24.0" customHeight="true">
+      <c r="A15" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B15" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C15" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D15" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E15" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F15" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H15" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I15" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J15" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K15" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L15" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M15" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O15" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P15" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R15" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S15" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T15" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="24.0" customHeight="true">
+      <c r="A16" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B16" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C16" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D16" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E16" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F16" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H16" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I16" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J16" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K16" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L16" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M16" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O16" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P16" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R16" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S16" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T16" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="24.0" customHeight="true">
+      <c r="A17" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B17" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C17" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D17" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F17" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H17" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I17" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J17" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K17" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L17" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M17" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O17" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P17" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R17" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S17" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T17" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="24.0" customHeight="true">
+      <c r="A18" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B18" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C18" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D18" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F18" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H18" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I18" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J18" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K18" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L18" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M18" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O18" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P18" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R18" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S18" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T18" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="24.0" customHeight="true">
+      <c r="A19" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="B19" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="C19" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="D19" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="F19" t="s" s="12">
+        <v>0</v>
+      </c>
+      <c r="H19" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="I19" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="J19" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="K19" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="L19" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="M19" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="O19" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="P19" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="R19" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="S19" t="s" s="13">
+        <v>0</v>
+      </c>
+      <c r="T19" t="s" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="24.0" customHeight="true"/>
+    <row r="21" ht="24.0" customHeight="true">
+      <c r="A21" t="s" s="8">
+        <v>47</v>
+      </c>
+      <c r="B21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="C21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="D21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="F21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H21" t="s" s="8">
+        <v>48</v>
+      </c>
+      <c r="I21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="M21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="O21" t="s" s="8">
+        <v>49</v>
+      </c>
+      <c r="P21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="R21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="S21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="T21" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="U21" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="24.0" customHeight="true">
+      <c r="A22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="B22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="C22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="D22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="E22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="F22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="M22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="O22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="P22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="R22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="S22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="T22" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="U22" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="24.0" customHeight="true">
+      <c r="A23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="B23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="C23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="D23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="F23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="M23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="O23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="P23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="R23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="S23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="T23" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="U23" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" ht="24.0" customHeight="true"/>
+    <row r="25" ht="24.0" customHeight="true">
+      <c r="A25" t="s" s="8">
+        <v>50</v>
+      </c>
+      <c r="B25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="C25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="D25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="F25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="G25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="M25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="N25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="O25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="P25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="R25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="S25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="T25" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="U25" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="24.0" customHeight="true">
+      <c r="A26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="B26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="C26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="D26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="E26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="F26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="G26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="H26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="I26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="J26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="K26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="L26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="M26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="N26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="O26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="P26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="R26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="S26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="T26" t="s" s="8">
+        <v>0</v>
+      </c>
+      <c r="U26" t="s" s="8">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="28">
+    <mergeCell ref="A1:O2"/>
+    <mergeCell ref="P1:U2"/>
+    <mergeCell ref="A3:U4"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:M6"/>
+    <mergeCell ref="O6:U6"/>
+    <mergeCell ref="A7:A19"/>
+    <mergeCell ref="H7:H19"/>
+    <mergeCell ref="O7:O19"/>
+    <mergeCell ref="B7:B19"/>
+    <mergeCell ref="I7:I19"/>
+    <mergeCell ref="P7:P19"/>
+    <mergeCell ref="C7:C19"/>
+    <mergeCell ref="J7:J19"/>
+    <mergeCell ref="Q7:Q19"/>
+    <mergeCell ref="D7:D19"/>
+    <mergeCell ref="K7:K19"/>
+    <mergeCell ref="R7:R19"/>
+    <mergeCell ref="E7:E19"/>
+    <mergeCell ref="L7:L19"/>
+    <mergeCell ref="S7:S19"/>
+    <mergeCell ref="F7:F19"/>
+    <mergeCell ref="M7:M19"/>
+    <mergeCell ref="T7:T19"/>
+    <mergeCell ref="A21:F23"/>
+    <mergeCell ref="H21:M23"/>
+    <mergeCell ref="O21:U23"/>
+    <mergeCell ref="A25:U26"/>
+  </mergeCells>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>